<commit_message>
Correct IDs and map labels
</commit_message>
<xml_diff>
--- a/data/LanguageFamily.xlsx
+++ b/data/LanguageFamily.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/psav050/Documents/GitHub/sync-coop-song-speech/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B22E143-2CA2-1A4D-ABEA-287E084E83A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D16A69E3-8D19-3949-9EAF-6851B2B34EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3520" yWindow="760" windowWidth="26720" windowHeight="13600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1060" yWindow="940" windowWidth="26720" windowHeight="13600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Many Voices 2 languages" sheetId="7" r:id="rId1"/>
@@ -89,9 +89,6 @@
     <t>Spanish [Bogotá]</t>
   </si>
   <si>
-    <t>Bahasa Indonesian</t>
-  </si>
-  <si>
     <t>Te Reo Māori (Māori)</t>
   </si>
   <si>
@@ -161,22 +158,10 @@
     <t>Sinhala</t>
   </si>
   <si>
-    <t>Italian (Rome)</t>
-  </si>
-  <si>
-    <t>Italian (Padua)</t>
-  </si>
-  <si>
-    <t>Russian (Ekaterinburg)</t>
-  </si>
-  <si>
     <t>German [Innsbruck]</t>
   </si>
   <si>
     <t>Czech</t>
-  </si>
-  <si>
-    <t>Russian (London)</t>
   </si>
   <si>
     <t>IsiZulu (Zulu)
@@ -212,6 +197,21 @@
   </si>
   <si>
     <t>Thai</t>
+  </si>
+  <si>
+    <t>Bahasa Indonesia</t>
+  </si>
+  <si>
+    <t>Italian [Rome]</t>
+  </si>
+  <si>
+    <t>Italian [Padua]</t>
+  </si>
+  <si>
+    <t>Russian [Ekaterinburg]</t>
+  </si>
+  <si>
+    <t>Russian [London]</t>
   </si>
 </sst>
 </file>
@@ -447,12 +447,6 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -479,16 +473,22 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -773,41 +773,41 @@
     </row>
     <row r="2" spans="1:44" ht="13" x14ac:dyDescent="0.15"/>
     <row r="3" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="42" t="s">
+      <c r="A3" s="41" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="G3" s="42" t="s">
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="G3" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="42"/>
-      <c r="I3" s="42"/>
-      <c r="J3" s="42"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="41"/>
     </row>
     <row r="4" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="32" t="s">
-        <v>47</v>
+      <c r="B4" s="30" t="s">
+        <v>42</v>
       </c>
       <c r="C4" s="5"/>
       <c r="D4" s="28">
         <v>16</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="9">
         <v>33</v>
       </c>
-      <c r="H4" s="41" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
+      <c r="H4" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
     </row>
     <row r="5" spans="1:44" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
@@ -821,68 +821,68 @@
         <v>17</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F5" s="8"/>
-      <c r="G5" s="42" t="s">
+      <c r="G5" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
     </row>
     <row r="6" spans="1:44" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="40" t="s">
         <v>13</v>
       </c>
       <c r="C6" s="5"/>
-      <c r="D6" s="34">
+      <c r="D6" s="32">
         <v>18</v>
       </c>
-      <c r="E6" s="35" t="s">
-        <v>51</v>
-      </c>
-      <c r="F6" s="37"/>
+      <c r="E6" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="35"/>
       <c r="G6" s="10">
         <v>34</v>
       </c>
-      <c r="H6" s="31" t="s">
+      <c r="H6" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
     </row>
     <row r="7" spans="1:44" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="34">
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="32">
         <v>19</v>
       </c>
-      <c r="E7" s="35" t="s">
+      <c r="E7" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="36" t="s">
+      <c r="F7" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="42" t="s">
+      <c r="G7" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
+      <c r="H7" s="41"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="41"/>
     </row>
     <row r="8" spans="1:44" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>4</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="28">
@@ -891,8 +891,8 @@
       <c r="E8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="33" t="s">
-        <v>39</v>
+      <c r="F8" s="31" t="s">
+        <v>38</v>
       </c>
       <c r="G8" s="11">
         <v>35</v>
@@ -910,45 +910,45 @@
         <v>5</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C9" s="7"/>
-      <c r="D9" s="34">
+      <c r="D9" s="32">
         <v>21</v>
       </c>
-      <c r="E9" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="37"/>
-      <c r="G9" s="42" t="s">
+      <c r="E9" s="33" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="35"/>
+      <c r="G9" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="42"/>
-      <c r="I9" s="42"/>
-      <c r="J9" s="42"/>
+      <c r="H9" s="41"/>
+      <c r="I9" s="41"/>
+      <c r="J9" s="41"/>
       <c r="AB9" s="3"/>
       <c r="AC9" s="3"/>
     </row>
     <row r="10" spans="1:44" ht="12.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="42" t="s">
+      <c r="A10" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="42"/>
-      <c r="C10" s="42"/>
-      <c r="D10" s="38">
+      <c r="B10" s="41"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="36">
         <v>22</v>
       </c>
-      <c r="E10" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" s="40" t="s">
-        <v>52</v>
+      <c r="E10" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="38" t="s">
+        <v>47</v>
       </c>
       <c r="G10" s="12">
         <v>36</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I10" s="13"/>
       <c r="J10" s="21"/>
@@ -960,10 +960,10 @@
         <v>6</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="33" t="s">
-        <v>49</v>
+        <v>43</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>44</v>
       </c>
       <c r="D11" s="28">
         <v>23</v>
@@ -971,15 +971,15 @@
       <c r="E11" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="33" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="42" t="s">
+      <c r="F11" s="31" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="41"/>
+      <c r="J11" s="41"/>
       <c r="AB11" s="3"/>
       <c r="AC11" s="3"/>
     </row>
@@ -988,21 +988,21 @@
         <v>7</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" s="8"/>
       <c r="D12" s="28">
         <v>24</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="33"/>
+        <v>54</v>
+      </c>
+      <c r="F12" s="31"/>
       <c r="G12" s="14">
         <v>37</v>
       </c>
       <c r="H12" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I12" s="15"/>
       <c r="J12" s="15"/>
@@ -1014,21 +1014,21 @@
         <v>8</v>
       </c>
       <c r="B13" s="22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="28">
         <v>25</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="33"/>
+        <v>55</v>
+      </c>
+      <c r="F13" s="31"/>
       <c r="G13" s="14">
         <v>38</v>
       </c>
       <c r="H13" s="25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I13" s="15"/>
       <c r="J13" s="15"/>
@@ -1040,21 +1040,21 @@
         <v>9</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="28">
         <v>26</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="F14" s="33"/>
+        <v>21</v>
+      </c>
+      <c r="F14" s="31"/>
       <c r="G14" s="14">
         <v>39</v>
       </c>
       <c r="H14" s="25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I14" s="15"/>
       <c r="J14" s="15"/>
@@ -1066,21 +1066,21 @@
         <v>10</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" s="8"/>
-      <c r="D15" s="34">
+      <c r="D15" s="32">
         <v>27</v>
       </c>
-      <c r="E15" s="35" t="s">
+      <c r="E15" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="F15" s="36"/>
+      <c r="F15" s="34"/>
       <c r="G15" s="14">
         <v>40</v>
       </c>
       <c r="H15" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I15" s="15"/>
       <c r="J15" s="15"/>
@@ -1092,24 +1092,24 @@
         <v>11</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="28">
         <v>28</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="F16" s="33" t="s">
-        <v>55</v>
-      </c>
-      <c r="G16" s="42" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="G16" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="H16" s="42"/>
-      <c r="I16" s="42"/>
-      <c r="J16" s="42"/>
+      <c r="H16" s="41"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="41"/>
       <c r="AB16" s="3"/>
       <c r="AC16" s="3"/>
     </row>
@@ -1118,21 +1118,21 @@
         <v>12</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="28">
         <v>29</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" s="33"/>
+        <v>41</v>
+      </c>
+      <c r="F17" s="31"/>
       <c r="G17" s="17">
         <v>41</v>
       </c>
       <c r="H17" s="27" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="I17" s="16"/>
       <c r="J17" s="20"/>
@@ -1142,43 +1142,43 @@
         <v>13</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="28">
         <v>30</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="F18" s="33"/>
-      <c r="G18" s="42" t="s">
-        <v>25</v>
-      </c>
-      <c r="H18" s="42"/>
-      <c r="I18" s="42"/>
-      <c r="J18" s="42"/>
+        <v>51</v>
+      </c>
+      <c r="F18" s="31"/>
+      <c r="G18" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" s="41"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="41"/>
     </row>
     <row r="19" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="28">
         <v>14</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="28">
         <v>31</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="F19" s="33"/>
+        <v>56</v>
+      </c>
+      <c r="F19" s="31"/>
       <c r="G19" s="18">
         <v>42</v>
       </c>
-      <c r="H19" s="43" t="s">
-        <v>26</v>
+      <c r="H19" s="39" t="s">
+        <v>25</v>
       </c>
       <c r="I19" s="19"/>
       <c r="J19" s="19"/>
@@ -1188,21 +1188,21 @@
         <v>15</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C20" s="8"/>
       <c r="D20" s="28">
         <v>32</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="F20" s="33"/>
+        <v>57</v>
+      </c>
+      <c r="F20" s="31"/>
       <c r="G20" s="18">
         <v>43</v>
       </c>
-      <c r="H20" s="43" t="s">
-        <v>27</v>
+      <c r="H20" s="39" t="s">
+        <v>26</v>
       </c>
       <c r="I20" s="19"/>
       <c r="J20" s="19"/>
@@ -1251,17 +1251,17 @@
     <row r="46" spans="11:11" ht="13" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="G5:J5"/>
-    <mergeCell ref="G7:J7"/>
-    <mergeCell ref="G9:J9"/>
     <mergeCell ref="G11:J11"/>
     <mergeCell ref="G16:J16"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="G18:J18"/>
     <mergeCell ref="G3:J3"/>
     <mergeCell ref="H6:J6"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G9:J9"/>
     <mergeCell ref="A7:C7"/>
   </mergeCells>
   <phoneticPr fontId="6"/>

</xml_diff>